<commit_message>
fixing examples downstream application
</commit_message>
<xml_diff>
--- a/downstream_application/data/example_data_new_uncertainty.xlsx
+++ b/downstream_application/data/example_data_new_uncertainty.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/veronica/Documents/GitHub/neural-concepts-team-E/downstream_application/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{893D8830-C663-F742-8B74-FFB5F429EEEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44556395-3F1F-0F44-B8E8-FF5DC009DA89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -350,9 +350,6 @@
     <t>Although, we achieved higher margins during the first half of fiscal 2025, those margins eroded somewhat during the second half of the year, primarily due to the impact of tariffs. Since April 2025, we have been subject to a 15% tariff on all goods imported from Italy which was reduced to 10% as of February 22, 2026. While this reduction provides some near-term relief, U.S. tariff policy remains unpredictable, creating uncertainty around potential future margin impacts.</t>
   </si>
   <si>
-    <t>ALEUY</t>
-  </si>
-  <si>
     <t>Allegro.eu S.A.</t>
   </si>
   <si>
@@ -887,6 +884,9 @@
   </si>
   <si>
     <t>SON.LS</t>
+  </si>
+  <si>
+    <t>ALE.WA</t>
   </si>
 </sst>
 </file>
@@ -1630,7 +1630,7 @@
     </row>
     <row r="10" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>71</v>
@@ -1791,31 +1791,31 @@
     </row>
     <row r="15" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="G15" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="H15" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="I15" s="4" t="s">
         <v>108</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>109</v>
       </c>
       <c r="J15" s="4" t="s">
         <v>20</v>
@@ -1824,31 +1824,31 @@
     </row>
     <row r="16" spans="1:11" ht="160" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="C16" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E16" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="G16" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="H16" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="I16" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>116</v>
       </c>
       <c r="J16" s="4" t="s">
         <v>20</v>
@@ -1857,31 +1857,31 @@
     </row>
     <row r="17" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E17" s="4" t="s">
+      <c r="F17" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="G17" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="H17" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="I17" s="4" t="s">
         <v>122</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>123</v>
       </c>
       <c r="J17" s="4" t="s">
         <v>20</v>
@@ -1890,31 +1890,31 @@
     </row>
     <row r="18" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="C18" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E18" s="4" t="s">
+      <c r="F18" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="G18" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G18" s="5" t="s">
+      <c r="H18" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="I18" s="4" t="s">
         <v>129</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>130</v>
       </c>
       <c r="J18" s="4" t="s">
         <v>20</v>
@@ -1923,31 +1923,31 @@
     </row>
     <row r="19" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="C19" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E19" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E19" s="4" t="s">
+      <c r="F19" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="G19" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="H19" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="I19" s="4" t="s">
         <v>136</v>
-      </c>
-      <c r="I19" s="4" t="s">
-        <v>137</v>
       </c>
       <c r="J19" s="4" t="s">
         <v>20</v>
@@ -1971,16 +1971,16 @@
         <v>70</v>
       </c>
       <c r="F20" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="H20" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="G20" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="H20" s="4" t="s">
+      <c r="I20" s="4" t="s">
         <v>140</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>141</v>
       </c>
       <c r="J20" s="4" t="s">
         <v>12</v>
@@ -1989,31 +1989,31 @@
     </row>
     <row r="21" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="C21" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="F21" s="4" t="s">
+      <c r="G21" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="G21" s="5" t="s">
+      <c r="H21" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="H21" s="4" t="s">
+      <c r="I21" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>148</v>
       </c>
       <c r="J21" s="4" t="s">
         <v>20</v>
@@ -2022,31 +2022,31 @@
     </row>
     <row r="22" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="C22" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E22" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E22" s="4" t="s">
+      <c r="F22" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="G22" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="G22" s="5" t="s">
+      <c r="H22" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="I22" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>155</v>
       </c>
       <c r="J22" s="4" t="s">
         <v>20</v>
@@ -2055,29 +2055,29 @@
     </row>
     <row r="23" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="C23" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="F23" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D23" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="F23" s="4" t="s">
+      <c r="G23" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>159</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J23" s="4" t="s">
         <v>20</v>
@@ -2086,31 +2086,31 @@
     </row>
     <row r="24" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="C24" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E24" s="4" t="s">
+      <c r="F24" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="G24" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="G24" s="5" t="s">
+      <c r="H24" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="I24" s="4" t="s">
         <v>166</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>167</v>
       </c>
       <c r="J24" s="4" t="s">
         <v>20</v>
@@ -2119,31 +2119,31 @@
     </row>
     <row r="25" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="C25" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E25" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E25" s="4" t="s">
+      <c r="F25" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="G25" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="G25" s="5" t="s">
+      <c r="H25" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="I25" s="4" t="s">
         <v>173</v>
-      </c>
-      <c r="I25" s="4" t="s">
-        <v>174</v>
       </c>
       <c r="J25" s="4" t="s">
         <v>20</v>
@@ -2152,31 +2152,31 @@
     </row>
     <row r="26" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="C26" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E26" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D26" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>181</v>
-      </c>
       <c r="F26" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H26" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="I26" s="4" t="s">
         <v>175</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>176</v>
       </c>
       <c r="J26" s="4" t="s">
         <v>20</v>
@@ -2185,31 +2185,31 @@
     </row>
     <row r="27" spans="1:11" ht="176" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="C27" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D27" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E27" s="4" t="s">
+      <c r="F27" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="G27" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="G27" s="5" t="s">
+      <c r="H27" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="I27" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="I27" s="4" t="s">
-        <v>188</v>
       </c>
       <c r="J27" s="4" t="s">
         <v>12</v>
@@ -2218,29 +2218,29 @@
     </row>
     <row r="28" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="C28" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C28" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E28" s="4" t="s">
+      <c r="F28" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="F28" s="4" t="s">
-        <v>192</v>
-      </c>
       <c r="G28" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H28" s="4"/>
       <c r="I28" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J28" s="4" t="s">
         <v>20</v>
@@ -2249,31 +2249,31 @@
     </row>
     <row r="29" spans="1:11" ht="176" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="C29" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E29" s="4" t="s">
+      <c r="F29" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="G29" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="G29" s="5" t="s">
+      <c r="H29" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="H29" s="4" t="s">
+      <c r="I29" s="4" t="s">
         <v>200</v>
-      </c>
-      <c r="I29" s="4" t="s">
-        <v>201</v>
       </c>
       <c r="J29" s="4" t="s">
         <v>20</v>
@@ -2282,29 +2282,29 @@
     </row>
     <row r="30" spans="1:11" ht="272" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="C30" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E30" s="4" t="s">
+      <c r="F30" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="G30" s="5" t="s">
         <v>205</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J30" s="4" t="s">
         <v>20</v>
@@ -2313,29 +2313,29 @@
     </row>
     <row r="31" spans="1:11" ht="192" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="C31" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D31" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E31" s="4" t="s">
+      <c r="F31" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="G31" s="5" t="s">
         <v>211</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>212</v>
       </c>
       <c r="H31" s="4"/>
       <c r="I31" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="J31" s="4" t="s">
         <v>20</v>
@@ -2344,29 +2344,29 @@
     </row>
     <row r="32" spans="1:11" ht="350" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="C32" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E32" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="C32" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D32" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E32" s="4" t="s">
+      <c r="F32" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="G32" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="H32" s="4"/>
       <c r="I32" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="J32" s="4" t="s">
         <v>20</v>
@@ -2375,29 +2375,29 @@
     </row>
     <row r="33" spans="1:11" ht="208" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="C33" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E33" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="C33" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D33" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E33" s="4" t="s">
+      <c r="F33" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="G33" s="5" t="s">
         <v>223</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>224</v>
       </c>
       <c r="H33" s="4"/>
       <c r="I33" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="J33" s="4" t="s">
         <v>20</v>
@@ -2406,31 +2406,31 @@
     </row>
     <row r="34" spans="1:11" ht="288" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B34" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E34" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="C34" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D34" s="4">
-        <v>2025</v>
-      </c>
-      <c r="E34" s="4" t="s">
+      <c r="F34" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="G34" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="G34" s="5" t="s">
+      <c r="H34" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="H34" s="4" t="s">
+      <c r="I34" s="4" t="s">
         <v>230</v>
-      </c>
-      <c r="I34" s="4" t="s">
-        <v>231</v>
       </c>
       <c r="J34" s="4" t="s">
         <v>20</v>
@@ -2492,47 +2492,47 @@
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="176" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="6">
-        <v>2025</v>
-      </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>233</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>234</v>
       </c>
       <c r="J2" s="6" t="s">
         <v>12</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="208" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>13</v>
@@ -2541,56 +2541,56 @@
         <v>2025</v>
       </c>
       <c r="E3" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="G3" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>242</v>
-      </c>
       <c r="J3" s="6" t="s">
         <v>20</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="6">
-        <v>2025</v>
-      </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>246</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>247</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>12</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="144" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>251</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>252</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>13</v>
@@ -2599,115 +2599,115 @@
         <v>2024</v>
       </c>
       <c r="E5" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>254</v>
-      </c>
       <c r="G5" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>20</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="365" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="6">
-        <v>2025</v>
-      </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="H6" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>262</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="H6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>260</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>261</v>
       </c>
       <c r="J6" s="6" t="s">
         <v>12</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="6">
-        <v>2025</v>
-      </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="I7" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="G7" s="6" t="s">
-        <v>263</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="I7" s="6" t="s">
+      <c r="J7" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="J7" s="6" t="s">
-        <v>270</v>
-      </c>
       <c r="K7" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="6">
+        <v>2025</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="6">
-        <v>2025</v>
-      </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>